<commit_message>
Phase 2: GUI portfolio table and service layer
</commit_message>
<xml_diff>
--- a/output/Zain_Wealth_Manager_Pro_v1.xlsx
+++ b/output/Zain_Wealth_Manager_Pro_v1.xlsx
@@ -54,7 +54,7 @@
     <t>XIRR</t>
   </si>
   <si>
-    <t>9.41%</t>
+    <t>9.39%</t>
   </si>
   <si>
     <t>Health Score</t>
@@ -66,7 +66,7 @@
     <t>Dividend Yield</t>
   </si>
   <si>
-    <t>1.68%</t>
+    <t>1.15%</t>
   </si>
   <si>
     <t>Monthly Investment Plan</t>
@@ -120,7 +120,7 @@
     <t>Progress</t>
   </si>
   <si>
-    <t>1.54%</t>
+    <t>1.88%</t>
   </si>
   <si>
     <t>Years Remaining</t>
@@ -150,7 +150,7 @@
     <t>• Excellent portfolio health.</t>
   </si>
   <si>
-    <t>• Goal progress is 1.54%. Continue regular investing.</t>
+    <t>• Goal progress is 1.88%. Continue regular investing.</t>
   </si>
   <si>
     <t>• Dividend income is strong.</t>
@@ -381,19 +381,19 @@
     <t>Recommendation</t>
   </si>
   <si>
-    <t>24.59%</t>
+    <t>38.46%</t>
+  </si>
+  <si>
+    <t>Good</t>
+  </si>
+  <si>
+    <t>19.33%</t>
   </si>
   <si>
     <t>Average</t>
   </si>
   <si>
-    <t>23.69%</t>
-  </si>
-  <si>
-    <t>51.72%</t>
-  </si>
-  <si>
-    <t>Good</t>
+    <t>42.21%</t>
   </si>
   <si>
     <t>0.0%</t>
@@ -614,7 +614,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>37800</c:v>
+                  <c:v>72450</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>36422</c:v>
@@ -1232,7 +1232,7 @@
     </row>
     <row r="9" spans="2:9">
       <c r="B9" s="5">
-        <v>153742</v>
+        <v>188392</v>
       </c>
       <c r="C9" s="5"/>
       <c r="F9" s="3" t="s">
@@ -1264,7 +1264,7 @@
     </row>
     <row r="12" spans="2:9">
       <c r="B12" s="5">
-        <v>68422</v>
+        <v>99172</v>
       </c>
       <c r="C12" s="5"/>
       <c r="F12" s="3" t="s">
@@ -1290,7 +1290,7 @@
     </row>
     <row r="15" spans="2:9">
       <c r="B15" s="5">
-        <v>74222</v>
+        <v>108872</v>
       </c>
       <c r="C15" s="5"/>
     </row>
@@ -1302,7 +1302,7 @@
     </row>
     <row r="18" spans="2:12">
       <c r="B18" s="5">
-        <v>5800</v>
+        <v>9700</v>
       </c>
       <c r="C18" s="5"/>
       <c r="F18" s="2" t="s">
@@ -1326,7 +1326,7 @@
         <v>30</v>
       </c>
       <c r="G20" s="6">
-        <v>153742</v>
+        <v>188392</v>
       </c>
     </row>
     <row r="21" spans="2:12">
@@ -1417,7 +1417,7 @@
         <v>16</v>
       </c>
       <c r="L31">
-        <v>37800</v>
+        <v>72450</v>
       </c>
     </row>
     <row r="32" spans="2:12">
@@ -2496,7 +2496,7 @@
         <v>16</v>
       </c>
       <c r="B5" s="6">
-        <v>37800</v>
+        <v>72450</v>
       </c>
       <c r="C5" s="3" t="s">
         <v>119</v>
@@ -2516,7 +2516,7 @@
         <v>121</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -2527,10 +2527,10 @@
         <v>79520</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
     </row>
     <row r="8" spans="1:4">

</xml_diff>